<commit_message>
Final Restart & Run All on Colab T4; sync report with rerun timings
Notebook re-executed top to bottom (execution counts 1-10, no errors).
All losses, accuracies, F1, grad norms, best epochs and eval predictions
are identical to the previous run; only wall-clock time per epoch and
peak memory changed, so REPORT.md and two notebook comment cells now
quote the rerun values (and the final-config sigma 0.0045).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission_2A202602940/experiments.xlsx
+++ b/submission_2A202602940/experiments.xlsx
@@ -1660,10 +1660,10 @@
         <v>0.6646635558504729</v>
       </c>
       <c r="W2" s="33" t="n">
-        <v>1.32264597285</v>
+        <v>1.345666531700181</v>
       </c>
       <c r="X2" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y2" s="33" t="inlineStr">
         <is>
@@ -1785,10 +1785,10 @@
         <v>0.7612533557248951</v>
       </c>
       <c r="W3" s="33" t="n">
-        <v>1.343346739499953</v>
+        <v>1.340230807550051</v>
       </c>
       <c r="X3" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y3" s="33" t="inlineStr">
         <is>
@@ -1910,10 +1910,10 @@
         <v>0.816958152576888</v>
       </c>
       <c r="W4" s="33" t="n">
-        <v>1.286818645299945</v>
+        <v>1.331178692649928</v>
       </c>
       <c r="X4" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y4" s="33" t="inlineStr">
         <is>
@@ -2035,10 +2035,10 @@
         <v>0.8390357563558714</v>
       </c>
       <c r="W5" s="33" t="n">
-        <v>1.287717804700014</v>
+        <v>1.35536646405003</v>
       </c>
       <c r="X5" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y5" s="33" t="inlineStr">
         <is>
@@ -2160,10 +2160,10 @@
         <v>0.8573463639034842</v>
       </c>
       <c r="W6" s="33" t="n">
-        <v>1.28715709340006</v>
+        <v>1.369954987300025</v>
       </c>
       <c r="X6" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y6" s="33" t="inlineStr">
         <is>
@@ -2285,10 +2285,10 @@
         <v>0.8573463639034842</v>
       </c>
       <c r="W7" s="33" t="n">
-        <v>1.285396225350087</v>
+        <v>1.33916191785006</v>
       </c>
       <c r="X7" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y7" s="33" t="inlineStr">
         <is>
@@ -2414,10 +2414,10 @@
         <v>0.8617669186606722</v>
       </c>
       <c r="W8" s="33" t="n">
-        <v>1.286350551449982</v>
+        <v>1.340477243250098</v>
       </c>
       <c r="X8" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y8" s="33" t="inlineStr">
         <is>
@@ -2539,10 +2539,10 @@
         <v>0.863011712873356</v>
       </c>
       <c r="W9" s="33" t="n">
-        <v>1.283507461899967</v>
+        <v>1.331553621700004</v>
       </c>
       <c r="X9" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y9" s="33" t="inlineStr">
         <is>
@@ -2664,10 +2664,10 @@
         <v>0.8732805427363912</v>
       </c>
       <c r="W10" s="33" t="n">
-        <v>1.329347046599992</v>
+        <v>1.371565747950035</v>
       </c>
       <c r="X10" s="33" t="n">
-        <v>199.107421875</v>
+        <v>203.220703125</v>
       </c>
       <c r="Y10" s="33" t="inlineStr">
         <is>
@@ -2789,10 +2789,10 @@
         <v>0.8747267862419351</v>
       </c>
       <c r="W11" s="33" t="n">
-        <v>1.470160418549858</v>
+        <v>1.365957603550078</v>
       </c>
       <c r="X11" s="33" t="n">
-        <v>216.0595703125</v>
+        <v>219.6728515625</v>
       </c>
       <c r="Y11" s="33" t="inlineStr">
         <is>
@@ -2914,10 +2914,10 @@
         <v>0.8951844572262216</v>
       </c>
       <c r="W12" s="33" t="n">
-        <v>1.376971009974955</v>
+        <v>1.464109189524947</v>
       </c>
       <c r="X12" s="33" t="n">
-        <v>216.0595703125</v>
+        <v>219.6728515625</v>
       </c>
       <c r="Y12" s="33" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0.8873313573056126</v>
       </c>
       <c r="W13" s="33" t="n">
-        <v>1.346279654000045</v>
+        <v>1.385015471099973</v>
       </c>
       <c r="X13" s="33" t="n">
-        <v>216.0595703125</v>
+        <v>219.6728515625</v>
       </c>
       <c r="Y13" s="33" t="inlineStr">
         <is>
@@ -3168,10 +3168,10 @@
         <v>0.8875222990137986</v>
       </c>
       <c r="W14" s="33" t="n">
-        <v>1.366462826274915</v>
+        <v>1.347674460149938</v>
       </c>
       <c r="X14" s="33" t="n">
-        <v>216.0595703125</v>
+        <v>219.6728515625</v>
       </c>
       <c r="Y14" s="33" t="inlineStr">
         <is>

</xml_diff>